<commit_message>
Initial commit: OrangeHRM Selenium Automation Framework
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\git\repository\completeFrameworkByAutomationInsider\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\git\repository2\completeFrameworkByAutomationInsider\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6CE456-49DE-47DD-AEE2-D2BA13D4643A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC21880F-D323-47D2-8467-46DD9DA39883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10935" yWindow="1905" windowWidth="9555" windowHeight="7875" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>password</t>
   </si>
@@ -44,13 +44,16 @@
     <t>Admin</t>
   </si>
   <si>
-    <t>admin1</t>
-  </si>
-  <si>
-    <t>admin1234</t>
-  </si>
-  <si>
-    <t>invalidLoginData</t>
+    <t>wrong User</t>
+  </si>
+  <si>
+    <t>wrongPas</t>
+  </si>
+  <si>
+    <t>wronguse</t>
+  </si>
+  <si>
+    <t>wrong pasi</t>
   </si>
 </sst>
 </file>
@@ -407,14 +410,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{757D615E-4124-4AA8-BA9F-993E3070A314}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -422,7 +425,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -430,9 +433,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C5" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Save progress: commit current workspace changes
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\git\repository2\completeFrameworkByAutomationInsider\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC21880F-D323-47D2-8467-46DD9DA39883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{1DE3602E-FFD5-4058-BA4B-018726B472B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10935" yWindow="1905" windowWidth="9555" windowHeight="7875" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8670" yWindow="1950" windowWidth="9825" windowHeight="7875" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
     <sheet name="invalidLoginData" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="addEmployeeData" sheetId="3" r:id="rId3"/>
+    <sheet name="claimData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
   <si>
     <t>password</t>
   </si>
@@ -54,16 +55,78 @@
   </si>
   <si>
     <t>wrong pasi</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>middleName</t>
+  </si>
+  <si>
+    <t>userName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>Babirye</t>
+  </si>
+  <si>
+    <t>Nakyeyune</t>
+  </si>
+  <si>
+    <t>confirmPassword</t>
+  </si>
+  <si>
+    <t>0702959972@Sn</t>
+  </si>
+  <si>
+    <t>eventName</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>remarks</t>
+  </si>
+  <si>
+    <t>United States Dollar</t>
+  </si>
+  <si>
+    <t>ElianaBabirye2</t>
+  </si>
+  <si>
+    <t>Accommodation</t>
+  </si>
+  <si>
+    <t>Automated test claim submission</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF79ABFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -86,14 +149,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -448,9 +515,99 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96977CEA-9DE3-4573-BFD8-A89EE43684FA}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{A7A20A68-162B-4FF7-87F7-5A5F3241432B}"/>
+    <hyperlink ref="E2" r:id="rId2" xr:uid="{70DE6728-DF34-440D-AF68-4883DA2A6E62}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBE47D9B-675D-4165-8AAF-40F54671577E}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add ClaimsAssignment page and tests - Refactor ResetPassword to ClaimsAssignmentPage, add ClaimsAssignmentTest, update BaseClass configuration
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\git\repository2\completeFrameworkByAutomationInsider\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{1DE3602E-FFD5-4058-BA4B-018726B472B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C81C8F7-EE95-4FBE-B0C2-1144266C08C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8670" yWindow="1950" windowWidth="9825" windowHeight="7875" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8670" yWindow="1950" windowWidth="9825" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>password</t>
   </si>
@@ -51,12 +51,6 @@
     <t>wrongPas</t>
   </si>
   <si>
-    <t>wronguse</t>
-  </si>
-  <si>
-    <t>wrong pasi</t>
-  </si>
-  <si>
     <t>firstName</t>
   </si>
   <si>
@@ -96,13 +90,13 @@
     <t>United States Dollar</t>
   </si>
   <si>
+    <t>Accommodation</t>
+  </si>
+  <si>
+    <t>Automated test claim submission</t>
+  </si>
+  <si>
     <t>ElianaBabirye2</t>
-  </si>
-  <si>
-    <t>Accommodation</t>
-  </si>
-  <si>
-    <t>Automated test claim submission</t>
   </si>
 </sst>
 </file>
@@ -439,7 +433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.85546875" customWidth="1"/>
@@ -462,14 +456,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -477,7 +463,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{757D615E-4124-4AA8-BA9F-993E3070A314}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" customWidth="1"/>
@@ -498,14 +484,6 @@
       </c>
       <c r="B2" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -528,42 +506,42 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="B1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -587,24 +565,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
         <v>18</v>
-      </c>
-      <c r="B1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
         <v>21</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>